<commit_message>
update encoding dan seeding pasien
</commit_message>
<xml_diff>
--- a/src/Database/Seeders/data/documents/patient-data.xlsx
+++ b/src/Database/Seeders/data/documents/patient-data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Kalpa\ExportTemplate\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A98376CB-32E1-42CE-80E5-DE144B0A9FA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72F8F546-46A7-46CE-99FE-2DC61812A43A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{660892B7-0D49-4A3F-9E80-4B384BA4EBF9}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="53">
   <si>
     <t>JENIS KELAMIN</t>
   </si>
@@ -132,17 +132,89 @@
   </si>
   <si>
     <t>3501121908960000</t>
+  </si>
+  <si>
+    <t>TGL BERKUNJUNG</t>
+  </si>
+  <si>
+    <t>POLIKLINIK</t>
+  </si>
+  <si>
+    <t>SOAP</t>
+  </si>
+  <si>
+    <t>UMUM</t>
+  </si>
+  <si>
+    <t>ORTHOPEDI</t>
+  </si>
+  <si>
+    <t>SUNAT</t>
+  </si>
+  <si>
+    <t>KECANTIKAN</t>
+  </si>
+  <si>
+    <t>MATA</t>
+  </si>
+  <si>
+    <t>THT</t>
+  </si>
+  <si>
+    <t>INTERNIS</t>
+  </si>
+  <si>
+    <t>GIGI &amp; MULUT</t>
+  </si>
+  <si>
+    <t>KIA</t>
+  </si>
+  <si>
+    <t>LANSIA</t>
+  </si>
+  <si>
+    <t>VACCINE</t>
+  </si>
+  <si>
+    <t>PATOLOGI KLINIK</t>
+  </si>
+  <si>
+    <t>PATOLOGI ANATOMI</t>
+  </si>
+  <si>
+    <t>MCU</t>
+  </si>
+  <si>
+    <t>RADIOLOGI</t>
+  </si>
+  <si>
+    <t>RAWAT INAP</t>
+  </si>
+  <si>
+    <t>VK</t>
+  </si>
+  <si>
+    <t>UGD</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
+    <numFmt numFmtId="166" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -191,7 +263,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
@@ -221,6 +293,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
+      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -632,8 +708,8 @@
       <c r="M2" s="5"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="56YuxYJb4aa3uR8S+mlj96SJk/t7RlVnZAk1Pks+uiKAzAnw6Ikw/gIQXhF8yGlvWoRT9tgS1g6rMukVGEzwYQ==" saltValue="ihs+t3ftYI5bBxj+kt5HrA==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
-  <dataValidations xWindow="40" yWindow="254" count="4">
+  <sheetProtection algorithmName="SHA-512" hashValue="Th71U17c+Y9eGYLq/SIILRsHu1Lhp/e8ij8viuQqy2c4mOwjE2Ek1zMzWJoQhGXnPdB217YuFia19JC1Wcu2Rg==" saltValue="YKXVPEQCBpOZmbfvD+VoKA==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
+  <dataValidations xWindow="992" yWindow="219" count="4">
     <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Hint" prompt="Format Tanggal lahir isi dengan Tahun-Bulan-Hari dengan ketentuan YYYY-mm-dd" sqref="F2:F1048576" xr:uid="{D0E60F89-56C4-4794-A578-9D6667D87AAD}">
       <formula1>DATE(1900,1,1)</formula1>
       <formula2>TODAY()</formula2>
@@ -651,7 +727,7 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xWindow="40" yWindow="254" count="3">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xWindow="992" yWindow="219" count="3">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Info" prompt="Jenis kelamin dapat diisi dengan 'Male' atau 'Female'" xr:uid="{3DD10DE3-4256-454D-814E-5E9BBF8B398B}">
           <x14:formula1>
             <xm:f>'MASTER DATA'!$B$1:$C$1</xm:f>
@@ -678,23 +754,84 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{52782042-C760-4902-8537-4E1398A30742}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="22.28515625" style="6" customWidth="1"/>
+    <col min="2" max="2" width="21.28515625" style="6" customWidth="1"/>
+    <col min="3" max="3" width="17" style="6" customWidth="1"/>
+    <col min="4" max="4" width="86.42578125" style="6" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C2" s="11"/>
+    </row>
+  </sheetData>
+  <sheetProtection algorithmName="SHA-512" hashValue="w1OKxnxvunv3x0BbHREvk4XKlaOeRdEtrpGEixRpQlw7WmbuI2WPMqc4CPeB4yS4xUbvCZDVAranxxrc2NVAcA==" saltValue="FSfdlkoGlYQfyhgPyHH23w==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
+  <dataValidations count="1">
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Hint" prompt="Format Tanggal lahir isi dengan Tahun-Bulan-Hari dengan ketentuan YYYY-mm-dd" sqref="C2" xr:uid="{0D258ED9-CBE7-47D2-9E76-838BFB1CE499}">
+      <formula1>DATE(1900,1,1)</formula1>
+      <formula2>TODAY()</formula2>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{B0AAB604-9165-4ECF-8A6D-DA555A39A74D}">
+          <x14:formula1>
+            <xm:f>'MASTER DATA'!$B$3:$S$3</xm:f>
+          </x14:formula1>
+          <xm:sqref>C3:C1048576</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1A593D3-5CDC-41CD-8095-9DE984838757}">
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:S3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.140625" customWidth="1"/>
+    <col min="2" max="2" width="7" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="4.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="4" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="5.140625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="3.42578125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="4.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
@@ -704,8 +841,8 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A2" s="10" t="s">
         <v>5</v>
       </c>
       <c r="B2" t="s">
@@ -745,8 +882,67 @@
         <v>17</v>
       </c>
     </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A3" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="B3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C3" t="s">
+        <v>36</v>
+      </c>
+      <c r="D3" t="s">
+        <v>37</v>
+      </c>
+      <c r="E3" t="s">
+        <v>38</v>
+      </c>
+      <c r="F3" t="s">
+        <v>39</v>
+      </c>
+      <c r="G3" t="s">
+        <v>40</v>
+      </c>
+      <c r="H3" t="s">
+        <v>41</v>
+      </c>
+      <c r="I3" t="s">
+        <v>42</v>
+      </c>
+      <c r="J3" t="s">
+        <v>43</v>
+      </c>
+      <c r="K3" t="s">
+        <v>44</v>
+      </c>
+      <c r="L3" t="s">
+        <v>45</v>
+      </c>
+      <c r="M3" t="s">
+        <v>46</v>
+      </c>
+      <c r="N3" t="s">
+        <v>47</v>
+      </c>
+      <c r="O3" t="s">
+        <v>48</v>
+      </c>
+      <c r="P3" t="s">
+        <v>49</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>50</v>
+      </c>
+      <c r="R3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S3" t="s">
+        <v>52</v>
+      </c>
+    </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="mc26GWzm67bmLEguIxYoscHsz1VCZfFHICrmyEfGQbdemnfYrx+R9Ua4G3AlPlt1JhnDs+G5BlI++jqymYL3+A==" saltValue="VqzzTTy2stU44mIzzndYTg==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="jtVlFONGoyZzzIrxFa0N8jgxzszBEIh2NlurxKcSX2om3cP0enbA+U3xe0LfOxkaQ43CaOBGfEvnkZzfVzxcbw==" saltValue="NKT5vKbcLcoqjrUuVPFQWg==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
   <dataConsolidate/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>